<commit_message>
Bot-3 high vol pipeline: method A/B, GANN wiring, ATR regime fix
</commit_message>
<xml_diff>
--- a/atr_results/nifty_atr_2025-01-01_to_2026-02-20.xlsx
+++ b/atr_results/nifty_atr_2025-01-01_to_2026-02-20.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Uzair Khan\Desktop\nifty bot\vixbot-refactor\atr_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02713634-077D-4A20-B03F-992D719630C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24539622-0FE4-43F5-8F1E-37D588B72558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -107,7 +107,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,7 +459,7 @@
         <f>E2&gt;1.5</f>
         <v>0</v>
       </c>
-      <c r="G2" s="5" t="b">
+      <c r="G2" t="b">
         <f>E2&gt;1.3</f>
         <v>0</v>
       </c>
@@ -510,7 +509,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G4" s="5" t="b">
+      <c r="G4" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -535,7 +534,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G5" s="5" t="b">
+      <c r="G5" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -560,7 +559,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G6" s="5" t="b">
+      <c r="G6" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -585,7 +584,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G7" s="5" t="b">
+      <c r="G7" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -610,7 +609,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G8" s="5" t="b">
+      <c r="G8" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -635,7 +634,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G9" s="5" t="b">
+      <c r="G9" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -660,7 +659,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G10" s="5" t="b">
+      <c r="G10" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -685,7 +684,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G11" s="5" t="b">
+      <c r="G11" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -710,7 +709,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G12" s="5" t="b">
+      <c r="G12" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -735,7 +734,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G13" s="5" t="b">
+      <c r="G13" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -785,7 +784,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G15" s="5" t="b">
+      <c r="G15" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -810,7 +809,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G16" s="5" t="b">
+      <c r="G16" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -835,7 +834,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G17" s="5" t="b">
+      <c r="G17" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -860,7 +859,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G18" s="5" t="b">
+      <c r="G18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -885,7 +884,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G19" s="5" t="b">
+      <c r="G19" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -910,7 +909,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G20" s="5" t="b">
+      <c r="G20" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -935,7 +934,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G21" s="5" t="b">
+      <c r="G21" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -960,7 +959,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G22" s="5" t="b">
+      <c r="G22" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -985,7 +984,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G23" s="5" t="b">
+      <c r="G23" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1010,7 +1009,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G24" s="5" t="b">
+      <c r="G24" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1035,7 +1034,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G25" s="5" t="b">
+      <c r="G25" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1060,7 +1059,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G26" s="5" t="b">
+      <c r="G26" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1085,7 +1084,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G27" s="5" t="b">
+      <c r="G27" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1110,7 +1109,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G28" s="5" t="b">
+      <c r="G28" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1135,12 +1134,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G29" s="5" t="b">
+      <c r="G29" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>45699</v>
       </c>
@@ -1185,7 +1184,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G31" s="5" t="b">
+      <c r="G31" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1210,7 +1209,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G32" s="5" t="b">
+      <c r="G32" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1235,7 +1234,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G33" s="5" t="b">
+      <c r="G33" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1260,7 +1259,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G34" s="5" t="b">
+      <c r="G34" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1285,7 +1284,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G35" s="5" t="b">
+      <c r="G35" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1310,7 +1309,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G36" s="5" t="b">
+      <c r="G36" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1335,7 +1334,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G37" s="5" t="b">
+      <c r="G37" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1360,7 +1359,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G38" s="5" t="b">
+      <c r="G38" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1385,7 +1384,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G39" s="5" t="b">
+      <c r="G39" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1410,7 +1409,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G40" s="5" t="b">
+      <c r="G40" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1435,12 +1434,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G41" s="5" t="b">
+      <c r="G41" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>45716</v>
       </c>
@@ -1485,7 +1484,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G43" s="5" t="b">
+      <c r="G43" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1510,12 +1509,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G44" s="5" t="b">
+      <c r="G44" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>45721</v>
       </c>
@@ -1560,7 +1559,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G46" s="5" t="b">
+      <c r="G46" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1585,7 +1584,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G47" s="5" t="b">
+      <c r="G47" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1610,7 +1609,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G48" s="5" t="b">
+      <c r="G48" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1635,7 +1634,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G49" s="5" t="b">
+      <c r="G49" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1660,7 +1659,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G50" s="5" t="b">
+      <c r="G50" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1685,7 +1684,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G51" s="5" t="b">
+      <c r="G51" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1710,7 +1709,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G52" s="5" t="b">
+      <c r="G52" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1735,7 +1734,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G53" s="5" t="b">
+      <c r="G53" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1760,7 +1759,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G54" s="5" t="b">
+      <c r="G54" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1785,7 +1784,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G55" s="5" t="b">
+      <c r="G55" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1810,7 +1809,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G56" s="5" t="b">
+      <c r="G56" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1835,7 +1834,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G57" s="5" t="b">
+      <c r="G57" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1860,7 +1859,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G58" s="5" t="b">
+      <c r="G58" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1885,7 +1884,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G59" s="5" t="b">
+      <c r="G59" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1910,7 +1909,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G60" s="5" t="b">
+      <c r="G60" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1935,7 +1934,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G61" s="5" t="b">
+      <c r="G61" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1985,7 +1984,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G63" s="5" t="b">
+      <c r="G63" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2010,12 +2009,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G64" s="5" t="b">
+      <c r="G64" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>45751</v>
       </c>
@@ -2040,7 +2039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>45754</v>
       </c>
@@ -2085,7 +2084,7 @@
         <f t="shared" ref="F67:F130" si="2">E67&gt;1.5</f>
         <v>0</v>
       </c>
-      <c r="G67" s="5" t="b">
+      <c r="G67" t="b">
         <f t="shared" ref="G67:G130" si="3">E67&gt;1.3</f>
         <v>0</v>
       </c>
@@ -2110,7 +2109,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G68" s="5" t="b">
+      <c r="G68" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2135,7 +2134,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G69" s="5" t="b">
+      <c r="G69" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2160,7 +2159,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G70" s="5" t="b">
+      <c r="G70" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2185,12 +2184,12 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G71" s="5" t="b">
+      <c r="G71" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>45764</v>
       </c>
@@ -2235,7 +2234,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G73" s="5" t="b">
+      <c r="G73" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2260,7 +2259,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G74" s="5" t="b">
+      <c r="G74" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2285,7 +2284,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G75" s="5" t="b">
+      <c r="G75" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2310,7 +2309,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G76" s="5" t="b">
+      <c r="G76" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2335,7 +2334,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G77" s="5" t="b">
+      <c r="G77" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2360,7 +2359,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G78" s="5" t="b">
+      <c r="G78" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2385,7 +2384,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G79" s="5" t="b">
+      <c r="G79" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2410,7 +2409,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G80" s="5" t="b">
+      <c r="G80" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2435,7 +2434,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G81" s="5" t="b">
+      <c r="G81" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2460,7 +2459,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G82" s="5" t="b">
+      <c r="G82" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2485,7 +2484,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G83" s="5" t="b">
+      <c r="G83" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2510,7 +2509,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G84" s="5" t="b">
+      <c r="G84" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2535,7 +2534,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G85" s="5" t="b">
+      <c r="G85" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2560,7 +2559,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G86" s="5" t="b">
+      <c r="G86" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2590,7 +2589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>45790</v>
       </c>
@@ -2635,7 +2634,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G89" s="5" t="b">
+      <c r="G89" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2685,7 +2684,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G91" s="5" t="b">
+      <c r="G91" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2710,7 +2709,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G92" s="5" t="b">
+      <c r="G92" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2735,7 +2734,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G93" s="5" t="b">
+      <c r="G93" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2760,7 +2759,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G94" s="5" t="b">
+      <c r="G94" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2785,7 +2784,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G95" s="5" t="b">
+      <c r="G95" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2810,7 +2809,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G96" s="5" t="b">
+      <c r="G96" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2835,7 +2834,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G97" s="5" t="b">
+      <c r="G97" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2860,7 +2859,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G98" s="5" t="b">
+      <c r="G98" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2885,7 +2884,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G99" s="5" t="b">
+      <c r="G99" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2910,7 +2909,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G100" s="5" t="b">
+      <c r="G100" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2935,7 +2934,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G101" s="5" t="b">
+      <c r="G101" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2960,7 +2959,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G102" s="5" t="b">
+      <c r="G102" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2985,7 +2984,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G103" s="5" t="b">
+      <c r="G103" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3010,7 +3009,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G104" s="5" t="b">
+      <c r="G104" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3035,12 +3034,12 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G105" s="5" t="b">
+      <c r="G105" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>45814</v>
       </c>
@@ -3085,7 +3084,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G107" s="5" t="b">
+      <c r="G107" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3110,7 +3109,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G108" s="5" t="b">
+      <c r="G108" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3135,7 +3134,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G109" s="5" t="b">
+      <c r="G109" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3185,7 +3184,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G111" s="5" t="b">
+      <c r="G111" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3210,7 +3209,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G112" s="5" t="b">
+      <c r="G112" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3235,7 +3234,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G113" s="5" t="b">
+      <c r="G113" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3260,7 +3259,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G114" s="5" t="b">
+      <c r="G114" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3285,12 +3284,12 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G115" s="5" t="b">
+      <c r="G115" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>45828</v>
       </c>
@@ -3335,7 +3334,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G117" s="5" t="b">
+      <c r="G117" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3360,7 +3359,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G118" s="5" t="b">
+      <c r="G118" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3385,7 +3384,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G119" s="5" t="b">
+      <c r="G119" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3410,7 +3409,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G120" s="5" t="b">
+      <c r="G120" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3435,7 +3434,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G121" s="5" t="b">
+      <c r="G121" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3460,7 +3459,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G122" s="5" t="b">
+      <c r="G122" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3485,7 +3484,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G123" s="5" t="b">
+      <c r="G123" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3510,7 +3509,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G124" s="5" t="b">
+      <c r="G124" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3535,7 +3534,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G125" s="5" t="b">
+      <c r="G125" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3560,7 +3559,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G126" s="5" t="b">
+      <c r="G126" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3585,7 +3584,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G127" s="5" t="b">
+      <c r="G127" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3610,7 +3609,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G128" s="5" t="b">
+      <c r="G128" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3635,7 +3634,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G129" s="5" t="b">
+      <c r="G129" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3660,7 +3659,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G130" s="5" t="b">
+      <c r="G130" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3685,7 +3684,7 @@
         <f t="shared" ref="F131:F194" si="4">E131&gt;1.5</f>
         <v>0</v>
       </c>
-      <c r="G131" s="5" t="b">
+      <c r="G131" t="b">
         <f t="shared" ref="G131:G194" si="5">E131&gt;1.3</f>
         <v>0</v>
       </c>
@@ -3710,7 +3709,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G132" s="5" t="b">
+      <c r="G132" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3735,7 +3734,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G133" s="5" t="b">
+      <c r="G133" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3760,7 +3759,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G134" s="5" t="b">
+      <c r="G134" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3785,12 +3784,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G135" s="5" t="b">
+      <c r="G135" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="1">
         <v>45856</v>
       </c>
@@ -3815,7 +3814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
         <v>45859</v>
       </c>
@@ -3860,7 +3859,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G138" s="5" t="b">
+      <c r="G138" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3885,12 +3884,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G139" s="5" t="b">
+      <c r="G139" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="1">
         <v>45862</v>
       </c>
@@ -3935,7 +3934,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G141" s="5" t="b">
+      <c r="G141" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3960,7 +3959,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G142" s="5" t="b">
+      <c r="G142" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -3985,7 +3984,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G143" s="5" t="b">
+      <c r="G143" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4010,7 +4009,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G144" s="5" t="b">
+      <c r="G144" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4060,7 +4059,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G146" s="5" t="b">
+      <c r="G146" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4085,7 +4084,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G147" s="5" t="b">
+      <c r="G147" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4110,7 +4109,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G148" s="5" t="b">
+      <c r="G148" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4135,12 +4134,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G149" s="5" t="b">
+      <c r="G149" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="1">
         <v>45876</v>
       </c>
@@ -4185,7 +4184,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G151" s="5" t="b">
+      <c r="G151" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4210,7 +4209,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G152" s="5" t="b">
+      <c r="G152" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4235,7 +4234,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G153" s="5" t="b">
+      <c r="G153" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4260,7 +4259,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G154" s="5" t="b">
+      <c r="G154" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4285,7 +4284,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G155" s="5" t="b">
+      <c r="G155" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4310,7 +4309,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G156" s="5" t="b">
+      <c r="G156" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4335,7 +4334,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G157" s="5" t="b">
+      <c r="G157" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4360,7 +4359,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G158" s="5" t="b">
+      <c r="G158" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4385,7 +4384,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G159" s="5" t="b">
+      <c r="G159" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4410,7 +4409,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G160" s="5" t="b">
+      <c r="G160" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4435,7 +4434,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G161" s="5" t="b">
+      <c r="G161" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4460,7 +4459,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G162" s="5" t="b">
+      <c r="G162" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4485,7 +4484,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G163" s="5" t="b">
+      <c r="G163" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4510,7 +4509,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G164" s="5" t="b">
+      <c r="G164" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4535,7 +4534,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G165" s="5" t="b">
+      <c r="G165" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4560,7 +4559,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G166" s="5" t="b">
+      <c r="G166" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4585,12 +4584,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G167" s="5" t="b">
+      <c r="G167" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="1">
         <v>45904</v>
       </c>
@@ -4635,7 +4634,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G169" s="5" t="b">
+      <c r="G169" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4660,7 +4659,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G170" s="5" t="b">
+      <c r="G170" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4685,7 +4684,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G171" s="5" t="b">
+      <c r="G171" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4710,7 +4709,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G172" s="5" t="b">
+      <c r="G172" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4735,7 +4734,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G173" s="5" t="b">
+      <c r="G173" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4760,7 +4759,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G174" s="5" t="b">
+      <c r="G174" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4785,7 +4784,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G175" s="5" t="b">
+      <c r="G175" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4810,7 +4809,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G176" s="5" t="b">
+      <c r="G176" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4835,7 +4834,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G177" s="5" t="b">
+      <c r="G177" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4860,7 +4859,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G178" s="5" t="b">
+      <c r="G178" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4885,7 +4884,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G179" s="5" t="b">
+      <c r="G179" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4910,7 +4909,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G180" s="5" t="b">
+      <c r="G180" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4935,7 +4934,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G181" s="5" t="b">
+      <c r="G181" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -4960,12 +4959,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G182" s="5" t="b">
+      <c r="G182" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="1">
         <v>45925</v>
       </c>
@@ -5035,7 +5034,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G185" s="5" t="b">
+      <c r="G185" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5060,7 +5059,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G186" s="5" t="b">
+      <c r="G186" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5110,7 +5109,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G188" s="5" t="b">
+      <c r="G188" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5135,7 +5134,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G189" s="5" t="b">
+      <c r="G189" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5160,7 +5159,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G190" s="5" t="b">
+      <c r="G190" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5185,7 +5184,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G191" s="5" t="b">
+      <c r="G191" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5210,7 +5209,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G192" s="5" t="b">
+      <c r="G192" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5235,7 +5234,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G193" s="5" t="b">
+      <c r="G193" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -5260,12 +5259,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G194" s="5" t="b">
+      <c r="G194" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="1">
         <v>45944</v>
       </c>
@@ -5310,7 +5309,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G196" s="5" t="b">
+      <c r="G196" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5335,12 +5334,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G197" s="5" t="b">
+      <c r="G197" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" s="1">
         <v>45947</v>
       </c>
@@ -5385,7 +5384,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G199" s="5" t="b">
+      <c r="G199" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5410,7 +5409,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G200" s="5" t="b">
+      <c r="G200" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5435,7 +5434,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G201" s="5" t="b">
+      <c r="G201" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5460,7 +5459,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G202" s="5" t="b">
+      <c r="G202" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5485,7 +5484,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G203" s="5" t="b">
+      <c r="G203" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5510,7 +5509,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G204" s="5" t="b">
+      <c r="G204" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5535,7 +5534,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G205" s="5" t="b">
+      <c r="G205" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5560,7 +5559,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G206" s="5" t="b">
+      <c r="G206" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5585,7 +5584,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G207" s="5" t="b">
+      <c r="G207" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5610,7 +5609,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G208" s="5" t="b">
+      <c r="G208" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5635,7 +5634,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G209" s="5" t="b">
+      <c r="G209" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5660,7 +5659,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G210" s="5" t="b">
+      <c r="G210" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5685,7 +5684,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G211" s="5" t="b">
+      <c r="G211" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5710,12 +5709,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G212" s="5" t="b">
+      <c r="G212" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="1">
         <v>45972</v>
       </c>
@@ -5760,7 +5759,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G214" s="5" t="b">
+      <c r="G214" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5785,7 +5784,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G215" s="5" t="b">
+      <c r="G215" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5810,7 +5809,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G216" s="5" t="b">
+      <c r="G216" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5835,7 +5834,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G217" s="5" t="b">
+      <c r="G217" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5860,7 +5859,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G218" s="5" t="b">
+      <c r="G218" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5885,7 +5884,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G219" s="5" t="b">
+      <c r="G219" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5910,7 +5909,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G220" s="5" t="b">
+      <c r="G220" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5935,7 +5934,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G221" s="5" t="b">
+      <c r="G221" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5960,7 +5959,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G222" s="5" t="b">
+      <c r="G222" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -5985,7 +5984,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G223" s="5" t="b">
+      <c r="G223" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6035,7 +6034,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G225" s="5" t="b">
+      <c r="G225" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6060,7 +6059,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G226" s="5" t="b">
+      <c r="G226" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6085,7 +6084,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G227" s="5" t="b">
+      <c r="G227" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6110,7 +6109,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G228" s="5" t="b">
+      <c r="G228" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6135,7 +6134,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G229" s="5" t="b">
+      <c r="G229" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6160,7 +6159,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G230" s="5" t="b">
+      <c r="G230" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6185,12 +6184,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G231" s="5" t="b">
+      <c r="G231" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="1">
         <v>45999</v>
       </c>
@@ -6235,7 +6234,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G233" s="5" t="b">
+      <c r="G233" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6260,7 +6259,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G234" s="5" t="b">
+      <c r="G234" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6285,7 +6284,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G235" s="5" t="b">
+      <c r="G235" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6310,7 +6309,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G236" s="5" t="b">
+      <c r="G236" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6335,7 +6334,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G237" s="5" t="b">
+      <c r="G237" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6360,7 +6359,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G238" s="5" t="b">
+      <c r="G238" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6385,7 +6384,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G239" s="5" t="b">
+      <c r="G239" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6410,7 +6409,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G240" s="5" t="b">
+      <c r="G240" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6435,7 +6434,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G241" s="5" t="b">
+      <c r="G241" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6460,7 +6459,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G242" s="5" t="b">
+      <c r="G242" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6485,7 +6484,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G243" s="5" t="b">
+      <c r="G243" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6510,7 +6509,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G244" s="5" t="b">
+      <c r="G244" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6535,7 +6534,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G245" s="5" t="b">
+      <c r="G245" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6560,7 +6559,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G246" s="5" t="b">
+      <c r="G246" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6585,12 +6584,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G247" s="5" t="b">
+      <c r="G247" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="1">
         <v>46022</v>
       </c>
@@ -6635,12 +6634,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G249" s="5" t="b">
+      <c r="G249" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" s="1">
         <v>46024</v>
       </c>
@@ -6685,7 +6684,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G251" s="5" t="b">
+      <c r="G251" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6710,7 +6709,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G252" s="5" t="b">
+      <c r="G252" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6735,7 +6734,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G253" s="5" t="b">
+      <c r="G253" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6860,7 +6859,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G258" s="5" t="b">
+      <c r="G258" t="b">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -6885,7 +6884,7 @@
         <f t="shared" ref="F259:F284" si="8">E259&gt;1.5</f>
         <v>0</v>
       </c>
-      <c r="G259" s="5" t="b">
+      <c r="G259" t="b">
         <f t="shared" ref="G259:G284" si="9">E259&gt;1.3</f>
         <v>0</v>
       </c>
@@ -6910,7 +6909,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G260" s="5" t="b">
+      <c r="G260" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -6985,7 +6984,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G263" s="5" t="b">
+      <c r="G263" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7010,7 +7009,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G264" s="5" t="b">
+      <c r="G264" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7035,7 +7034,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G265" s="5" t="b">
+      <c r="G265" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7060,7 +7059,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G266" s="5" t="b">
+      <c r="G266" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7085,7 +7084,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G267" s="5" t="b">
+      <c r="G267" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7110,7 +7109,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G268" s="5" t="b">
+      <c r="G268" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7160,7 +7159,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G270" s="5" t="b">
+      <c r="G270" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7210,7 +7209,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G272" s="5" t="b">
+      <c r="G272" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7235,7 +7234,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G273" s="5" t="b">
+      <c r="G273" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7260,7 +7259,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G274" s="5" t="b">
+      <c r="G274" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7285,7 +7284,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G275" s="5" t="b">
+      <c r="G275" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7310,7 +7309,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G276" s="5" t="b">
+      <c r="G276" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7335,7 +7334,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G277" s="5" t="b">
+      <c r="G277" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7360,7 +7359,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G278" s="5" t="b">
+      <c r="G278" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7385,7 +7384,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G279" s="5" t="b">
+      <c r="G279" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7410,7 +7409,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G280" s="5" t="b">
+      <c r="G280" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7435,7 +7434,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G281" s="5" t="b">
+      <c r="G281" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7460,7 +7459,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G282" s="5" t="b">
+      <c r="G282" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -7510,14 +7509,14 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G284" s="5" t="b">
+      <c r="G284" t="b">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G284" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="6">
+    <filterColumn colId="5">
       <filters>
         <filter val="TRUE"/>
       </filters>

</xml_diff>